<commit_message>
Mapa com todas as macroatividades e ID com vários números por célula
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q51eCtHXwFCUfvUJ8nmQQ4
</commit_message>
<xml_diff>
--- a/roadmap_executivo_exemplo.xlsx
+++ b/roadmap_executivo_exemplo.xlsx
@@ -1481,7 +1481,7 @@
   <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -1534,9 +1534,9 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>M01</t>
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -1555,8 +1555,8 @@
       <c r="E2" s="3" t="n">
         <v>46297</v>
       </c>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
+      <c r="F2" s="4" t="inlineStr"/>
+      <c r="G2" s="4" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Sim</t>
@@ -1564,9 +1564,9 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>M02</t>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -1585,12 +1585,12 @@
       <c r="E3" s="3" t="n">
         <v>46304</v>
       </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>M01</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr"/>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr"/>
       <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Sim</t>
@@ -1598,9 +1598,9 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>M03</t>
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>30</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -1619,12 +1619,12 @@
       <c r="E4" s="3" t="n">
         <v>46318</v>
       </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>M02</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Não</t>
@@ -1632,9 +1632,9 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>M04</t>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>40</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -1653,12 +1653,12 @@
       <c r="E5" s="3" t="n">
         <v>46325</v>
       </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>M03</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr"/>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Não</t>
@@ -1666,9 +1666,9 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>M05</t>
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>50; 51</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -1687,12 +1687,12 @@
       <c r="E6" s="3" t="n">
         <v>46353</v>
       </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>M04</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr"/>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr"/>
       <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Não</t>
@@ -1700,9 +1700,9 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>M06</t>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>60</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -1721,12 +1721,12 @@
       <c r="E7" s="3" t="n">
         <v>46360</v>
       </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>M05</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr"/>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr"/>
       <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Não</t>
@@ -1734,9 +1734,9 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>M07</t>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>70</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1755,8 +1755,8 @@
       <c r="E8" s="3" t="n">
         <v>46325</v>
       </c>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
+      <c r="F8" s="4" t="inlineStr"/>
+      <c r="G8" s="4" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Não</t>
@@ -1764,9 +1764,9 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>M08</t>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>80</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1785,12 +1785,12 @@
       <c r="E9" s="3" t="n">
         <v>46360</v>
       </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>M07</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr"/>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Não</t>
@@ -1798,9 +1798,9 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>M09</t>
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>90; 91</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1819,12 +1819,12 @@
       <c r="E10" s="3" t="n">
         <v>46395</v>
       </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>M08</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr"/>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Não</t>
@@ -1832,9 +1832,9 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>M10</t>
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>100</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1853,8 +1853,8 @@
       <c r="E11" s="3" t="n">
         <v>46318</v>
       </c>
-      <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr"/>
+      <c r="F11" s="4" t="inlineStr"/>
+      <c r="G11" s="4" t="inlineStr"/>
       <c r="H11" s="2" t="inlineStr">
         <is>
           <t>Não</t>
@@ -1862,9 +1862,9 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>M11</t>
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>110</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1883,12 +1883,12 @@
       <c r="E12" s="3" t="n">
         <v>46339</v>
       </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>M10; M04</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr"/>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>100; 40</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr"/>
       <c r="H12" s="2" t="inlineStr">
         <is>
           <t>Não</t>
@@ -1896,9 +1896,9 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>M12</t>
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>120; 121; 122</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1917,12 +1917,12 @@
       <c r="E13" s="3" t="n">
         <v>46367</v>
       </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>M11; M05</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr"/>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>110; 51</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr"/>
       <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Não</t>
@@ -1930,9 +1930,9 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>M13</t>
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>130</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1951,12 +1951,12 @@
       <c r="E14" s="3" t="n">
         <v>46387</v>
       </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>M12</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr"/>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>122</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr"/>
       <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Não</t>
@@ -1964,9 +1964,9 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>M14</t>
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>140</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1985,12 +1985,12 @@
       <c r="E15" s="3" t="n">
         <v>46416</v>
       </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>M13; M09</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr"/>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>130; 91</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr"/>
       <c r="H15" s="2" t="inlineStr">
         <is>
           <t>Não</t>
@@ -1998,9 +1998,9 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>M15</t>
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>150</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -2019,8 +2019,8 @@
       <c r="E16" s="3" t="n">
         <v>46297</v>
       </c>
-      <c r="F16" s="2" t="inlineStr"/>
-      <c r="G16" s="2" t="inlineStr"/>
+      <c r="F16" s="4" t="inlineStr"/>
+      <c r="G16" s="4" t="inlineStr"/>
       <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Sim</t>
@@ -2028,9 +2028,9 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>M16</t>
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>160</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -2049,12 +2049,12 @@
       <c r="E17" s="3" t="n">
         <v>46304</v>
       </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>M15</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr"/>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr"/>
       <c r="H17" s="2" t="inlineStr">
         <is>
           <t>Sim</t>
@@ -2062,9 +2062,9 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>M17</t>
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>170</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -2083,12 +2083,12 @@
       <c r="E18" s="3" t="n">
         <v>46309</v>
       </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>M16</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr"/>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>160</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr"/>
       <c r="H18" s="2" t="inlineStr">
         <is>
           <t>Não</t>
@@ -2096,9 +2096,9 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>M18</t>
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>180</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -2117,12 +2117,12 @@
       <c r="E19" s="3" t="n">
         <v>46318</v>
       </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>M17</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr"/>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>170</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr"/>
       <c r="H19" s="2" t="inlineStr">
         <is>
           <t>Não</t>
@@ -2130,9 +2130,9 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>M19</t>
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>190; 191</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -2151,12 +2151,12 @@
       <c r="E20" s="3" t="n">
         <v>46379</v>
       </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>M18; M06</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr"/>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>180; 60</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr"/>
       <c r="H20" s="2" t="inlineStr">
         <is>
           <t>Não</t>
@@ -2164,9 +2164,9 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>M20</t>
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>200</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -2185,8 +2185,8 @@
       <c r="E21" s="3" t="n">
         <v>46304</v>
       </c>
-      <c r="F21" s="2" t="inlineStr"/>
-      <c r="G21" s="2" t="inlineStr"/>
+      <c r="F21" s="4" t="inlineStr"/>
+      <c r="G21" s="4" t="inlineStr"/>
       <c r="H21" s="2" t="inlineStr">
         <is>
           <t>Sim</t>
@@ -2194,9 +2194,9 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>M21</t>
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>210</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2215,12 +2215,12 @@
       <c r="E22" s="3" t="n">
         <v>46318</v>
       </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>M20; M02</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr"/>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>200; 20</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr"/>
       <c r="H22" s="2" t="inlineStr">
         <is>
           <t>Não</t>
@@ -2228,9 +2228,9 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>M22</t>
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>220</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -2249,12 +2249,12 @@
       <c r="E23" s="3" t="n">
         <v>46379</v>
       </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>M21; M06; M17</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr"/>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>210; 60; 170</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr"/>
       <c r="H23" s="2" t="inlineStr">
         <is>
           <t>Não</t>
@@ -2280,7 +2280,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -2396,39 +2396,46 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Cada linha vira um losango na raia da frente, na DataFim. O retângulo da frente vai da menor DataInicio à maior DataFim.</t>
+          <t>ID: um ou mais números separados por ponto e vírgula (ex.: 01; 50; 90) — uma macroatividade pode reunir várias atividades. Predecessoras/Sucessoras citam esses números.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
+          <t>Cada linha vira um losango na raia da frente, na DataFim. O retângulo da frente vai da menor DataInicio à maior DataFim.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
           <t>Frente sem nenhuma iniciativa aparece como 'Sem cronograma · data-alvo'.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr"/>
-    </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+      <c r="A21" s="5" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>Calculado pelo painel (não preencher): frentes sem cronograma, dependências em risco, frentes com pendência, bloqueios de prontidão, status dos marcos e carga de marcos por semana.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>Dependência em risco: se comprovada, quando alguma predecessora está atrasada ou a sucessora começa antes de ela terminar; se hipótese, quando a frente que entrega está sem cronograma, tem Bloqueio, risco Alto ou marco atrasado.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr"/>
-    </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="A24" s="5" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>Não renomeie as tabelas nem as colunas: o fluxo do Power Automate depende delas. Dados desta planilha são fictícios.</t>
         </is>

</xml_diff>

<commit_message>
Detalhe da frente, evolução e pontos críticos (tbPontos) e prontidão recolhível
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q51eCtHXwFCUfvUJ8nmQQ4
</commit_message>
<xml_diff>
--- a/roadmap_executivo_exemplo.xlsx
+++ b/roadmap_executivo_exemplo.xlsx
@@ -10,7 +10,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Painel" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frentes" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Iniciativas" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruções" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pontos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruções" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -164,9 +165,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tbPainel" displayName="tbPainel" ref="A1:G2" headerRowCount="1">
-  <autoFilter ref="A1:G2"/>
-  <tableColumns count="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tbPainel" displayName="tbPainel" ref="A1:H2" headerRowCount="1">
+  <autoFilter ref="A1:H2"/>
+  <tableColumns count="8">
     <tableColumn id="1" name="Pergunta"/>
     <tableColumn id="2" name="Veredito"/>
     <tableColumn id="3" name="PrazoFinal"/>
@@ -174,15 +175,16 @@
     <tableColumn id="5" name="DependenciasEmRisco"/>
     <tableColumn id="6" name="FrentesComPendencia"/>
     <tableColumn id="7" name="BloqueiosProntidao"/>
+    <tableColumn id="8" name="TituloEvolucao"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tbFrentes" displayName="tbFrentes" ref="A1:S9" headerRowCount="1">
-  <autoFilter ref="A1:S9"/>
-  <tableColumns count="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tbFrentes" displayName="tbFrentes" ref="A1:AA9" headerRowCount="1">
+  <autoFilter ref="A1:AA9"/>
+  <tableColumns count="27">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Frente"/>
     <tableColumn id="3" name="Lider"/>
@@ -202,15 +204,23 @@
     <tableColumn id="17" name="RiscoDescricao"/>
     <tableColumn id="18" name="RecebeDe"/>
     <tableColumn id="19" name="EntregaPara"/>
+    <tableColumn id="20" name="NomeCurto"/>
+    <tableColumn id="21" name="Descricao"/>
+    <tableColumn id="22" name="Area"/>
+    <tableColumn id="23" name="Sponsor"/>
+    <tableColumn id="24" name="EscopoComentario"/>
+    <tableColumn id="25" name="PrazoComentario"/>
+    <tableColumn id="26" name="EntregaveisComentario"/>
+    <tableColumn id="27" name="RecursosComentario"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tbIniciativas" displayName="tbIniciativas" ref="A1:H23" headerRowCount="1">
-  <autoFilter ref="A1:H23"/>
-  <tableColumns count="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tbIniciativas" displayName="tbIniciativas" ref="A1:J23" headerRowCount="1">
+  <autoFilter ref="A1:J23"/>
+  <tableColumns count="10">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Macroatividade"/>
     <tableColumn id="3" name="Frente"/>
@@ -219,6 +229,27 @@
     <tableColumn id="6" name="Predecessoras"/>
     <tableColumn id="7" name="Sucessoras"/>
     <tableColumn id="8" name="Concluida"/>
+    <tableColumn id="9" name="Responsavel"/>
+    <tableColumn id="10" name="Avanco"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tbPontos" displayName="tbPontos" ref="A1:J16" headerRowCount="1">
+  <autoFilter ref="A1:J16"/>
+  <tableColumns count="10">
+    <tableColumn id="1" name="Tipo"/>
+    <tableColumn id="2" name="Titulo"/>
+    <tableColumn id="3" name="Descricao"/>
+    <tableColumn id="4" name="Acao"/>
+    <tableColumn id="5" name="Frente"/>
+    <tableColumn id="6" name="Responsavel"/>
+    <tableColumn id="7" name="Prazo"/>
+    <tableColumn id="8" name="Criticidade"/>
+    <tableColumn id="9" name="Data"/>
+    <tableColumn id="10" name="Fonte"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -513,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -523,6 +554,7 @@
     <col width="21" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="56" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -561,6 +593,11 @@
           <t>BloqueiosProntidao</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>TituloEvolucao</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -580,6 +617,11 @@
       <c r="E2" s="4" t="n"/>
       <c r="F2" s="4" t="n"/>
       <c r="G2" s="4" t="n"/>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>Desde a última diretiva: o que avançou e o que ainda trava jan/27</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -600,7 +642,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S9"/>
+  <dimension ref="A1:AA9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -622,6 +664,14 @@
     <col width="50" customWidth="1" min="17" max="17"/>
     <col width="16" customWidth="1" min="18" max="18"/>
     <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="50" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="16" customWidth="1" min="23" max="23"/>
+    <col width="40" customWidth="1" min="24" max="24"/>
+    <col width="40" customWidth="1" min="25" max="25"/>
+    <col width="40" customWidth="1" min="26" max="26"/>
+    <col width="40" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -720,6 +770,46 @@
           <t>EntregaPara</t>
         </is>
       </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>NomeCurto</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Descricao</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Sponsor</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>EscopoComentario</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>PrazoComentario</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>EntregaveisComentario</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>RecursosComentario</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -809,6 +899,46 @@
           <t>02</t>
         </is>
       </c>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>Dados</t>
+        </is>
+      </c>
+      <c r="U2" s="5" t="inlineStr">
+        <is>
+          <t>Validação das fontes de dados de clientes e disponibilização para o motor.</t>
+        </is>
+      </c>
+      <c r="V2" s="2" t="inlineStr">
+        <is>
+          <t>Dados</t>
+        </is>
+      </c>
+      <c r="W2" s="2" t="inlineStr">
+        <is>
+          <t>Marcos Vieira</t>
+        </is>
+      </c>
+      <c r="X2" s="5" t="inlineStr">
+        <is>
+          <t>Fontes principais validadas; faltam 2 bases secundárias.</t>
+        </is>
+      </c>
+      <c r="Y2" s="5" t="inlineStr">
+        <is>
+          <t>Validação vence em 23/10; consolidação em 27/11.</t>
+        </is>
+      </c>
+      <c r="Z2" s="5" t="inlineStr">
+        <is>
+          <t>5 macroatividades com datas; 2 concluídas.</t>
+        </is>
+      </c>
+      <c r="AA2" s="2" t="inlineStr">
+        <is>
+          <t>Todas as áreas alocadas.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -902,6 +1032,46 @@
           <t>04; 05; 06; 07</t>
         </is>
       </c>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>Motor</t>
+        </is>
+      </c>
+      <c r="U3" s="5" t="inlineStr">
+        <is>
+          <t>Motor de regras que calcula a elegibilidade e o benefício.</t>
+        </is>
+      </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>Tecnologia</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="inlineStr">
+        <is>
+          <t>Marcos Vieira</t>
+        </is>
+      </c>
+      <c r="X3" s="2" t="inlineStr">
+        <is>
+          <t>Regras de exceção em discussão.</t>
+        </is>
+      </c>
+      <c r="Y3" s="2" t="inlineStr">
+        <is>
+          <t>Depende da base validada (frente 01).</t>
+        </is>
+      </c>
+      <c r="Z3" s="2" t="inlineStr">
+        <is>
+          <t>Entregáveis mapeados e datados.</t>
+        </is>
+      </c>
+      <c r="AA3" s="2" t="inlineStr">
+        <is>
+          <t>CRM e Preço com alocação parcial.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -991,6 +1161,46 @@
           <t>05; 06; 07</t>
         </is>
       </c>
+      <c r="T4" s="2" t="inlineStr">
+        <is>
+          <t>Portfólio</t>
+        </is>
+      </c>
+      <c r="U4" s="5" t="inlineStr">
+        <is>
+          <t>Definição do novo portfólio de serviços e sua carga nos sistemas.</t>
+        </is>
+      </c>
+      <c r="V4" s="2" t="inlineStr">
+        <is>
+          <t>Produtos</t>
+        </is>
+      </c>
+      <c r="W4" s="2" t="inlineStr">
+        <is>
+          <t>Luísa Campos</t>
+        </is>
+      </c>
+      <c r="X4" s="2" t="inlineStr">
+        <is>
+          <t>Escopo fechado.</t>
+        </is>
+      </c>
+      <c r="Y4" s="2" t="inlineStr">
+        <is>
+          <t>Data final comprometida.</t>
+        </is>
+      </c>
+      <c r="Z4" s="2" t="inlineStr">
+        <is>
+          <t>Entregáveis mapeados.</t>
+        </is>
+      </c>
+      <c r="AA4" s="2" t="inlineStr">
+        <is>
+          <t>Time de dados sem alocação confirmada.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1084,6 +1294,46 @@
           <t>08</t>
         </is>
       </c>
+      <c r="T5" s="2" t="inlineStr">
+        <is>
+          <t>Parceiro</t>
+        </is>
+      </c>
+      <c r="U5" s="5" t="inlineStr">
+        <is>
+          <t>Integração com parceiro externo para informar elegibilidade.</t>
+        </is>
+      </c>
+      <c r="V5" s="2" t="inlineStr">
+        <is>
+          <t>Parcerias</t>
+        </is>
+      </c>
+      <c r="W5" s="2" t="inlineStr">
+        <is>
+          <t>Luísa Campos</t>
+        </is>
+      </c>
+      <c r="X5" s="5" t="inlineStr">
+        <is>
+          <t>Escopo mínimo ainda não acordado com o parceiro.</t>
+        </is>
+      </c>
+      <c r="Y5" s="2" t="inlineStr">
+        <is>
+          <t>Sem cronograma do parceiro.</t>
+        </is>
+      </c>
+      <c r="Z5" s="2" t="inlineStr">
+        <is>
+          <t>Requisitos em levantamento.</t>
+        </is>
+      </c>
+      <c r="AA5" s="2" t="inlineStr">
+        <is>
+          <t>Equipe do parceiro não confirmada.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1177,6 +1427,46 @@
           <t>08</t>
         </is>
       </c>
+      <c r="T6" s="2" t="inlineStr">
+        <is>
+          <t>Cobrança</t>
+        </is>
+      </c>
+      <c r="U6" s="5" t="inlineStr">
+        <is>
+          <t>Adaptação do sistema de cobrança para aplicar o novo benefício.</t>
+        </is>
+      </c>
+      <c r="V6" s="2" t="inlineStr">
+        <is>
+          <t>Tecnologia</t>
+        </is>
+      </c>
+      <c r="W6" s="2" t="inlineStr">
+        <is>
+          <t>Marcos Vieira</t>
+        </is>
+      </c>
+      <c r="X6" s="2" t="inlineStr">
+        <is>
+          <t>Escopo fechado.</t>
+        </is>
+      </c>
+      <c r="Y6" s="2" t="inlineStr">
+        <is>
+          <t>Janela de congelamento reduz testes.</t>
+        </is>
+      </c>
+      <c r="Z6" s="2" t="inlineStr">
+        <is>
+          <t>Entregáveis mapeados.</t>
+        </is>
+      </c>
+      <c r="AA6" s="2" t="inlineStr">
+        <is>
+          <t>Áreas alocadas.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1270,6 +1560,46 @@
           <t>08</t>
         </is>
       </c>
+      <c r="T7" s="2" t="inlineStr">
+        <is>
+          <t>Cliente</t>
+        </is>
+      </c>
+      <c r="U7" s="5" t="inlineStr">
+        <is>
+          <t>Jornada e comunicação do benefício para o cliente.</t>
+        </is>
+      </c>
+      <c r="V7" s="2" t="inlineStr">
+        <is>
+          <t>Canais</t>
+        </is>
+      </c>
+      <c r="W7" s="2" t="inlineStr">
+        <is>
+          <t>Paula Moraes</t>
+        </is>
+      </c>
+      <c r="X7" s="2" t="inlineStr">
+        <is>
+          <t>Canal do MVP em decisão.</t>
+        </is>
+      </c>
+      <c r="Y7" s="2" t="inlineStr">
+        <is>
+          <t>Lançamento depende do motor.</t>
+        </is>
+      </c>
+      <c r="Z7" s="2" t="inlineStr">
+        <is>
+          <t>Telas finais em andamento.</t>
+        </is>
+      </c>
+      <c r="AA7" s="2" t="inlineStr">
+        <is>
+          <t>Áreas alocadas.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1363,6 +1693,46 @@
           <t>08</t>
         </is>
       </c>
+      <c r="T8" s="2" t="inlineStr">
+        <is>
+          <t>Atendente</t>
+        </is>
+      </c>
+      <c r="U8" s="5" t="inlineStr">
+        <is>
+          <t>Ferramentas e treinamento da rede de atendimento.</t>
+        </is>
+      </c>
+      <c r="V8" s="2" t="inlineStr">
+        <is>
+          <t>Canais</t>
+        </is>
+      </c>
+      <c r="W8" s="2" t="inlineStr">
+        <is>
+          <t>Paula Moraes</t>
+        </is>
+      </c>
+      <c r="X8" s="2" t="inlineStr">
+        <is>
+          <t>Escopo mínimo em aberto.</t>
+        </is>
+      </c>
+      <c r="Y8" s="2" t="inlineStr">
+        <is>
+          <t>Treinamento concorre com campanhas.</t>
+        </is>
+      </c>
+      <c r="Z8" s="2" t="inlineStr">
+        <is>
+          <t>Roteiro em andamento.</t>
+        </is>
+      </c>
+      <c r="AA8" s="2" t="inlineStr">
+        <is>
+          <t>Preço com alocação parcial.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1452,6 +1822,46 @@
         </is>
       </c>
       <c r="S9" s="2" t="inlineStr"/>
+      <c r="T9" s="2" t="inlineStr">
+        <is>
+          <t>Conciliação</t>
+        </is>
+      </c>
+      <c r="U9" s="5" t="inlineStr">
+        <is>
+          <t>Gestão e conciliação financeira do benefício.</t>
+        </is>
+      </c>
+      <c r="V9" s="2" t="inlineStr">
+        <is>
+          <t>Operações</t>
+        </is>
+      </c>
+      <c r="W9" s="2" t="inlineStr">
+        <is>
+          <t>Paula Moraes</t>
+        </is>
+      </c>
+      <c r="X9" s="2" t="inlineStr">
+        <is>
+          <t>Sem dono definido.</t>
+        </is>
+      </c>
+      <c r="Y9" s="2" t="inlineStr">
+        <is>
+          <t>Sem cronograma.</t>
+        </is>
+      </c>
+      <c r="Z9" s="2" t="inlineStr">
+        <is>
+          <t>Sem entregáveis mapeados.</t>
+        </is>
+      </c>
+      <c r="AA9" s="2" t="inlineStr">
+        <is>
+          <t>Áreas não confirmadas.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="3">
@@ -1478,7 +1888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1489,6 +1899,8 @@
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1532,6 +1944,16 @@
           <t>Concluida</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Responsavel</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Avanco</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -1562,6 +1984,16 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Dados · Engenharia</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -1596,6 +2028,16 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Dados · Engenharia</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -1630,6 +2072,16 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Dados · Engenharia</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -1664,6 +2116,16 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Tecnologia · Motor</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1698,6 +2160,12 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Tecnologia · Motor</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1732,6 +2200,12 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Tecnologia · Motor</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1762,6 +2236,16 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Produtos</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>80%</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1796,6 +2280,12 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Produtos</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1830,6 +2320,12 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Produtos</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1860,6 +2356,16 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Tecnologia · Cobrança</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1894,6 +2400,12 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Tecnologia · Cobrança</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1928,6 +2440,12 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Tecnologia · Cobrança</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1962,6 +2480,12 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Tecnologia · Cobrança</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1996,6 +2520,12 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Tecnologia · Cobrança</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -2026,6 +2556,16 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Canais · UX</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -2060,6 +2600,16 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Canais · UX</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -2094,6 +2644,16 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Canais · UX</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>70%</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -2128,6 +2688,12 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Canais · UX</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -2162,6 +2728,12 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Canais · UX</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -2192,6 +2764,16 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Canais · Rede</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -2226,6 +2808,16 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Canais · Rede</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -2260,6 +2852,12 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Canais · Rede</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -2280,7 +2878,676 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:J16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Descricao</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Acao</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Frente</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Responsavel</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Prazo</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Criticidade</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Fonte</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Evolução</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Governança e visão integrada</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Rotina de acompanhamento 3x por semana e fórum quinzenal; macroatividades padronizadas por frente.</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>PMO</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="3" t="n">
+        <v>46311</v>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Reunião de acompanhamento</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Evolução</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Base de clientes</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Fontes principais validadas; faltam 2 bases secundárias.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Ana Ribeiro</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="n"/>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="3" t="n">
+        <v>46311</v>
+      </c>
+      <c r="J3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Evolução</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Motor de regras</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Arquitetura definida; ingestão passa a depender da base validada.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Mendes</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="n"/>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="3" t="n">
+        <v>46309</v>
+      </c>
+      <c r="J4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Evolução</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Portfólio</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Pesquisa de nomes concluída, sem fechamento; comissão em 03/11.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Julia Prado</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="3" t="n">
+        <v>46310</v>
+      </c>
+      <c r="J5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Evolução</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Cliente e atendente</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Proposta de canal mínimo apresentada; escopo do atendente em discussão.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>06; 07</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Diego Martins</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="n"/>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="3" t="n">
+        <v>46311</v>
+      </c>
+      <c r="J6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Evolução</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Gestão e conciliação</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Frente passou a ter uma única atividade, ainda sem responsável.</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Fernanda Rocha</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="3" t="n">
+        <v>46311</v>
+      </c>
+      <c r="J7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Risco</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Canal do MVP: decisão hoje</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Proposta de canal mínimo com cobertura parcial da carteira; canal alternativo exige esforço maior.</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Decidir entre canal mínimo ou condicionar o alternativo à análise de esforço.</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>03; 06; 07</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Diego Martins</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="n"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Reunião de 16/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Risco</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Parceiro sem previsibilidade</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Macroatividades do parceiro sem datas; requisitos fecham em 30/10.</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Fixar escopo mínimo e responsáveis; entregar requisitos e esforço até 30/10.</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>04; 02; 08</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Rafael Lima</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>46325</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="n"/>
+      <c r="J9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Risco</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Mensagens 2 e 3 sem dono</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Só a primeira mensagem tem esforço confirmado; as demais dependem do motor.</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Definir quem constrói as mensagens 2 e 3 e o responsável pelo front.</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>06; 02; 05</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Beatriz Alves</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>46316</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="n"/>
+      <c r="J10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Risco</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Nome do portfólio trava 8 atividades</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Campo obrigatório sem fechamento; trava comissão, materiais e ofertas.</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Fechar o nome e levar à comissão.</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>03; 02; 06; 07</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Julia Prado</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="n"/>
+      <c r="J11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Risco</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Calendários motor × cobrança</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Cobrança homologa em dezembro e depende da base no ambiente de dados.</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Alinhar arquitetura, data de apuração e agenda de testes integrados.</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>02; 05</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Mendes</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>46325</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="n"/>
+      <c r="J12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Atenção</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Qualidade de 2 bases secundárias</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Aderência caiu para 50–60%; tratado como ponto de atenção, não bloqueio.</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Investigar a mudança de regra com Engenharia e Produtos.</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Ana Ribeiro</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="n"/>
+      <c r="J13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Pendência</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Consolidar bases de investimento</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Consolidação exige esforço técnico elevado, sem prazo de refatoração.</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Engenharia estrutura a visão consolidada e o monitoramento de carga.</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Engenharia</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>46352</v>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="3" t="n"/>
+      <c r="J14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Pendência</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Regra de elegibilidade não fechada</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Regra pode exigir débito técnico se não for aprovada antes da rotina.</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Aprovar a regra antes da rotina de elegibilidade.</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>01; 02</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Ana Ribeiro</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>a definir</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="3" t="n"/>
+      <c r="J15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Pendência</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Escopo mínimo do atendente</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Escopo segue em aberto e a capacidade da equipe não foi estimada.</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Fechar o mínimo e priorizar a capacidade.</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Diego Martins</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>46314</v>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="3" t="n"/>
+      <c r="J16" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="A2:A500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Evolução,Pendência,Atenção,Risco"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Crítico,Alto,Médio,Baixo"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -2420,22 +3687,63 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Calculado pelo painel (não preencher): frentes sem cronograma, dependências em risco, frentes com pendência, bloqueios de prontidão, status dos marcos e carga de marcos por semana.</t>
+          <t>tbPontos (aba Pontos) — preenchida à mão</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
+          <t>Tipo: Evolução (cartões 'o que avançou'), Pendência ou Atenção (aparecem no detalhe da frente e Atenção também nos pontos críticos) ou Risco (cartões de pontos críticos).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Titulo e Descricao: o que aconteceu / qual é o risco. Acao: plano de ação ou decisão necessária. Frente: IDs separados por ; ou 'Todas'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Responsavel e Prazo (data ou texto como 'a definir'). Criticidade: Crítico, Alto, Médio ou Baixo (agrupa os cartões). Data: data da evolução. Fonte: opcional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Campos opcionais do detalhe: na tbFrentes, NomeCurto, Descricao, Area, Sponsor e os comentários de prontidão; na tbIniciativas, Responsavel e Avanco (%). Vazio = a tela só não mostra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Calculado pelo painel (não preencher): frentes sem cronograma, dependências em risco, frentes com pendência, bloqueios de prontidão, status dos marcos e carga de marcos por semana.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
           <t>Dependência em risco: se comprovada, quando alguma predecessora está atrasada ou a sucessora começa antes de ela terminar; se hipótese, quando a frente que entrega está sem cronograma, tem Bloqueio, risco Alto ou marco atrasado.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>Não renomeie as tabelas nem as colunas: o fluxo do Power Automate depende delas. Dados desta planilha são fictícios.</t>
         </is>

</xml_diff>

<commit_message>
Status da macroatividade pelo % de avanço
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q51eCtHXwFCUfvUJ8nmQQ4
</commit_message>
<xml_diff>
--- a/roadmap_executivo_exemplo.xlsx
+++ b/roadmap_executivo_exemplo.xlsx
@@ -3547,7 +3547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A32"/>
+  <dimension ref="A1:A33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -3723,27 +3723,34 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="5" t="inlineStr"/>
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Status da macroatividade pelo Avanco (%): 100% = Concluído; abaixo de 100% com DataFim vencida = Atrasado; 1% a 99% = Em andamento; 0% = Não iniciado. Com Avanco vazio, vale a coluna Concluida e as datas.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="6" t="inlineStr">
+      <c r="A29" s="5" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>Calculado pelo painel (não preencher): frentes sem cronograma, dependências em risco, frentes com pendência, bloqueios de prontidão, status dos marcos e carga de marcos por semana.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>Dependência em risco: se comprovada, quando alguma predecessora está atrasada ou a sucessora começa antes de ela terminar; se hipótese, quando a frente que entrega está sem cronograma, tem Bloqueio, risco Alto ou marco atrasado.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr"/>
-    </row>
     <row r="32">
-      <c r="A32" s="6" t="inlineStr">
+      <c r="A32" s="5" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
         <is>
           <t>Não renomeie as tabelas nem as colunas: o fluxo do Power Automate depende delas. Dados desta planilha são fictícios.</t>
         </is>

</xml_diff>

<commit_message>
Veredito só com os 3 estados em destaque; tela renomeada para Evoluções e roadblocks
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q51eCtHXwFCUfvUJ8nmQQ4
</commit_message>
<xml_diff>
--- a/roadmap_executivo_exemplo.xlsx
+++ b/roadmap_executivo_exemplo.xlsx
@@ -617,9 +617,9 @@
       <c r="E2" s="4" t="n"/>
       <c r="F2" s="4" t="n"/>
       <c r="G2" s="4" t="n"/>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>Desde a última diretiva: o que avançou e o que ainda trava jan/27</t>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Evoluções e roadblocks</t>
         </is>
       </c>
     </row>
@@ -3694,7 +3694,7 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Tipo: Evolução (cartões 'o que avançou'), Pendência ou Atenção (aparecem no detalhe da frente e Atenção também nos pontos críticos) ou Risco (cartões de pontos críticos).</t>
+          <t>Tipo: Evolução (bloco Evoluções), Pendência ou Atenção (aparecem no detalhe da frente e Atenção também nos roadblocks) ou Risco (roadblocks).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Roadblocks incluem Pendência, com etiqueta de tipo (Risco, Atenção, Pendência)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q51eCtHXwFCUfvUJ8nmQQ4
</commit_message>
<xml_diff>
--- a/roadmap_executivo_exemplo.xlsx
+++ b/roadmap_executivo_exemplo.xlsx
@@ -3483,7 +3483,11 @@
           <t>a definir</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
       <c r="I15" s="3" t="n"/>
       <c r="J15" s="2" t="inlineStr"/>
     </row>
@@ -3694,7 +3698,7 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Tipo: Evolução (bloco Evoluções), Pendência ou Atenção (aparecem no detalhe da frente e Atenção também nos roadblocks) ou Risco (roadblocks).</t>
+          <t>Tipo: Evolução (bloco Evoluções); Risco, Atenção e Pendência viram roadblocks (com etiqueta do tipo). Pendência e Atenção também aparecem no detalhe da frente. Na tabela de roadblocks entram os de Criticidade Crítico ou Alto; os demais vão para o rodapé.</t>
         </is>
       </c>
     </row>

</xml_diff>